<commit_message>
Add shared Datalund suite sample workbook
Generate one Projects+Tasks Excel as the suite source of truth, refresh
per-visual sample extracts from it, and link the suite file from home
and product pages.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/GanttSampleData.xlsx
+++ b/public/downloads/GanttSampleData.xlsx
@@ -52,11 +52,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,16 +421,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,22 +477,22 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46027</v>
+        <v>46184</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46036</v>
-      </c>
-      <c r="E2" s="3" t="n">
+        <v>46198</v>
+      </c>
+      <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Discovery</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Alex</t>
+          <t>Ada Ng</t>
         </is>
       </c>
     </row>
@@ -504,204 +503,568 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46034</v>
+        <v>46193</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>46043</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0.85</v>
+        <v>46208</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Discovery</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Jordan Lee</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>API Design</t>
+          <t>API design</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46037</v>
+        <v>46204</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>46051</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>0.6</v>
+        <v>46223</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.75</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>Sam Ortiz</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>FAT prep</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>46044</v>
+        <v>46254</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>0.35</v>
+        <v>46270</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.2</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Ada Ng</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Cable survey</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>46044</v>
+        <v>46154</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>0.45</v>
+        <v>46188</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>Bo Berg</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Alpha Gate</t>
+          <t>Cable pull</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>46065</v>
+        <v>46204</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>1</v>
+        <v>46254</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.4</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alex</t>
+          <t>Bo Berg</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>Weather hold</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="D8" t="n">
-        <v>14</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>0.1</v>
+        <v>46244</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Riley</t>
+          <t>Riley Chen</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Scope workshop</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>46072</v>
+        <v>46214</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>46079</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>0</v>
+        <v>46228</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Initiation</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alex</t>
+          <t>Cara Diaz</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Go-Live</t>
+          <t>Budget review</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>46082</v>
+        <v>46223</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>46082</v>
-      </c>
-      <c r="E10" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Initiation</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Finn Olsen</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Scope freeze</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Launch</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Alex</t>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Initiation</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Cara Diaz</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Model training</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46124</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Dan Okonkwo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Sam Ortiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>46245</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Ada Ng</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Evidence gather</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Operate</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Eva Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Audit prep</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Operate</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Eva Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Permit draft</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Finn Olsen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Stakeholder map</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>46254</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Jordan Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Roster closeout</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Operate</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Ada Ng</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Data cleanse</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Bo Berg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Model v1</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Dan Okonkwo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>QA soak</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>46254</v>
+      </c>
+      <c r="D22" t="n">
+        <v>14</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Riley Chen</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>On-call week</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Operate</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Bo Berg</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Vendor RFP</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Eva Holm</t>
         </is>
       </c>
     </row>
@@ -716,18 +1079,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Power BI Desktop test data for the custom Gantt visual</t>
-        </is>
-      </c>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Power BI Desktop test data for DataLund Gantt chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -739,21 +1105,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. Import GanttChart.pbiviz (Visualizations … → Import a visual from a file).</t>
+          <t>2. Import ganttChart.pbiviz (Visualizations … → Import a visual from a file).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Bind: Task→Task, Start Date→Start, End Date→End, Duration→Duration (optional extras: Progress, Group, Resource).</t>
+          <t>3. Bind: Task→Task, Start Date→Start, End Date→End, Duration→Duration (optional: Progress, Group, Resource).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alpha Gate and Go-Live are zero-duration milestones. QA uses Duration instead of End.</t>
+          <t>Scope freeze is a zero-duration milestone. QA soak uses Duration instead of End.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>For the full suite (Task List + Resource Load on one page), use DatalundSuiteSample.xlsx.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ship latest suite visuals from GitHub main
Pull branded .pbiviz builds prepared for AppSource packaging:
Gantt 1.9.1.0, Resource Load 1.0.0.0 refresh, Task List 1.0.3.0 refresh.
Rebuild DataLundSuite.zip, sync starter Excels, and bump changelog /
SoftwareApplication version metadata.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/GanttSampleData.xlsx
+++ b/public/downloads/GanttSampleData.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="0&quot;%&quot;"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -126,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -145,8 +146,14 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -513,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="82" customWidth="1" min="1" max="1"/>
@@ -566,35 +573,21 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>3. Bind Task, Start Date, End Date — then Group, Resource</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Resource well → Resource (assignee). Do not put Project in Resource.</t>
-        </is>
-      </c>
-    </row>
+          <t>3. Bind Task, Start Date, End Date — then Progress, Group, Resource</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Progress is optional later for bar fill — not in this starter.</t>
+          <t>Same columns as Resource Load. Full suite page → DatalundSuiteSample.xlsx</t>
         </is>
       </c>
     </row>
     <row r="10"/>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Same columns as Resource Load. Full suite page → DatalundSuiteSample.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>https://datalund.no/visuals/gantt/</t>
         </is>
@@ -606,7 +599,7 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -619,14 +612,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -647,10 +641,15 @@
       </c>
       <c r="D1" s="9" t="inlineStr">
         <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>Resource</t>
         </is>
@@ -668,35 +667,41 @@
       <c r="C2" s="11" t="n">
         <v>46198</v>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="F2" s="10" t="inlineStr">
         <is>
           <t>Ada Ng</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>API design</t>
         </is>
       </c>
-      <c r="B3" s="13" t="n">
+      <c r="B3" s="14" t="n">
         <v>46204</v>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="14" t="n">
         <v>46223</v>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="15" t="n">
+        <v>75</v>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
         <is>
           <t>Sam Ortiz</t>
         </is>
@@ -714,35 +719,41 @@
       <c r="C4" s="11" t="n">
         <v>46270</v>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Ada Ng</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Cable pull</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="14" t="n">
         <v>46204</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>46254</v>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Bo Berg</t>
         </is>
@@ -760,35 +771,41 @@
       <c r="C6" s="11" t="n">
         <v>46252</v>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Riley Chen</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>On-call week</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="14" t="n">
         <v>46252</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>46258</v>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>Bo Berg</t>
         </is>
@@ -806,35 +823,41 @@
       <c r="C8" s="11" t="n">
         <v>46228</v>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Cara Diaz</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Scope freeze</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="14" t="n">
         <v>46246</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>46246</v>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Cara Diaz</t>
         </is>
@@ -852,35 +875,41 @@
       <c r="C10" s="11" t="n">
         <v>46244</v>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="12" t="n">
+        <v>85</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Sam Ortiz</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="14" t="n">
         <v>46245</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>46259</v>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Ada Ng</t>
         </is>
@@ -898,42 +927,48 @@
       <c r="C12" s="11" t="n">
         <v>46296</v>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>Plan</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>Finn Olsen</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Stakeholder map</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="14" t="n">
         <v>46254</v>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>Plan</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Jordan Lee</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:F13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>